<commit_message>
data: 更新 2025-08 (TT=162.222 Kwai=67.623)
</commit_message>
<xml_diff>
--- a/docs/data/巴西数据底稿_2025-08.xlsx
+++ b/docs/data/巴西数据底稿_2025-08.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M74"/>
+  <dimension ref="A1:O86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -439,6 +439,8 @@
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -464,81 +466,97 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>短剧</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>社区</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>新闻资讯</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>在线阅读</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>浏览器/搜索</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>音乐/音频</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>游戏</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>电商</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>生活服务</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>AI</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="B2" t="n">
-        <v>404.11</v>
+        <v>403.47</v>
       </c>
       <c r="C2" t="n">
-        <v>483.02</v>
+        <v>483.03</v>
       </c>
       <c r="D2" t="n">
         <v>1.59</v>
       </c>
       <c r="E2" t="n">
-        <v>280.04</v>
+        <v>278.62</v>
       </c>
       <c r="F2" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="G2" t="n">
         <v>16.38</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>0.71</v>
       </c>
-      <c r="H2" t="n">
-        <v>8</v>
-      </c>
       <c r="I2" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="J2" t="n">
         <v>95.44</v>
       </c>
-      <c r="J2" t="n">
-        <v>22.81</v>
-      </c>
       <c r="K2" t="n">
+        <v>22.76</v>
+      </c>
+      <c r="L2" t="n">
         <v>129.51</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>30.17</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>7.8</v>
+      </c>
+      <c r="O2" t="n">
+        <v>27.62</v>
       </c>
     </row>
     <row r="3">
@@ -608,7 +626,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>162.221</v>
+        <v>162.222</v>
       </c>
     </row>
     <row r="11">
@@ -734,435 +752,541 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Waze</t>
+          <t>ReelShort</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>9.039999999999999</v>
+        <v>0.8090000000000001</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Pinterest</t>
+          <t>DramaBox - movies and drama</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>5.969</v>
+        <v>0.605</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Reddit</t>
+          <t>GoodShort</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>1.367</v>
+        <v>0.316</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Quora</t>
+          <t>ShortTV</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0.007</v>
+        <v>0.068</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Helo - Share Your Life</t>
+          <t>eStory- short dramas &amp; Novel</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0</v>
+        <v>0.029</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Google News</t>
+          <t>Waze</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>0.181</v>
+        <v>9.039999999999999</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>Pinterest</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>0.14</v>
+        <v>5.969</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>UOL | Notícias em Tempo Real</t>
+          <t>Reddit</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>0.067</v>
+        <v>1.367</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Opera News</t>
+          <t>Quora</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>0.053</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Folha de S.Paulo</t>
+          <t>Helo - Share Your Life</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Wattpad</t>
+          <t>Google News</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>2.226</v>
+        <v>0.181</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Kindle</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>1.117</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>JW Library</t>
+          <t>UOL | Notícias em Tempo Real</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>0.898</v>
+        <v>0.067</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>GALATEA</t>
+          <t>Opera News</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>0.506</v>
+        <v>0.053</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ReadEra by READERA LLC</t>
+          <t>Folha de S.Paulo</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>0.433</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Chrome Browser</t>
+          <t>Wattpad</t>
         </is>
       </c>
       <c r="I44" t="n">
-        <v>67.696</v>
+        <v>2.226</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Kindle</t>
         </is>
       </c>
       <c r="I45" t="n">
-        <v>16.825</v>
+        <v>1.117</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Brave Browser: Fast AdBlocker</t>
+          <t>JW Library</t>
         </is>
       </c>
       <c r="I46" t="n">
-        <v>3.017</v>
+        <v>0.898</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Samsung Internet Browser</t>
+          <t>GALATEA</t>
         </is>
       </c>
       <c r="I47" t="n">
-        <v>2.064</v>
+        <v>0.506</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Opera Browser</t>
+          <t>ReadEra by READERA LLC</t>
         </is>
       </c>
       <c r="I48" t="n">
-        <v>1.808</v>
+        <v>0.433</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Spotify</t>
+          <t>Chrome Browser</t>
         </is>
       </c>
       <c r="J50" t="n">
-        <v>11.045</v>
+        <v>67.696</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>YouTube Music</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="J51" t="n">
-        <v>5.116</v>
+        <v>16.825</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Lark Player</t>
+          <t>Brave Browser: Fast AdBlocker</t>
         </is>
       </c>
       <c r="J52" t="n">
-        <v>1.039</v>
+        <v>3.017</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Mi Music</t>
+          <t>Samsung Internet Browser</t>
         </is>
       </c>
       <c r="J53" t="n">
-        <v>0.516</v>
+        <v>2.064</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>RadiosNet</t>
+          <t>Opera Browser</t>
         </is>
       </c>
       <c r="J54" t="n">
-        <v>0.409</v>
+        <v>1.808</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ROBLOX</t>
+          <t>Spotify</t>
         </is>
       </c>
       <c r="K56" t="n">
-        <v>53.431</v>
+        <v>11.045</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Free Fire</t>
+          <t>YouTube Music</t>
         </is>
       </c>
       <c r="K57" t="n">
-        <v>5.564</v>
+        <v>5.116</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Clash Royale</t>
+          <t>Lark Player</t>
         </is>
       </c>
       <c r="K58" t="n">
-        <v>3.351</v>
+        <v>1.039</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Brawl Stars</t>
+          <t>Mi Music</t>
         </is>
       </c>
       <c r="K59" t="n">
-        <v>3.317</v>
+        <v>0.516</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Minecraft Pocket Edition</t>
+          <t>RadiosNet</t>
         </is>
       </c>
       <c r="K60" t="n">
-        <v>2.948</v>
+        <v>0.409</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Shopee</t>
+          <t>ROBLOX</t>
         </is>
       </c>
       <c r="L62" t="n">
-        <v>14.57</v>
+        <v>53.431</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>MercadoLibre</t>
+          <t>Free Fire</t>
         </is>
       </c>
       <c r="L63" t="n">
-        <v>5.876</v>
+        <v>5.564</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>SHEIN</t>
+          <t>Clash Royale</t>
         </is>
       </c>
       <c r="L64" t="n">
-        <v>2.96</v>
+        <v>3.351</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>AliExpress</t>
+          <t>Brawl Stars</t>
         </is>
       </c>
       <c r="L65" t="n">
-        <v>1.362</v>
+        <v>3.317</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Temu</t>
+          <t>Minecraft Pocket Edition</t>
         </is>
       </c>
       <c r="L66" t="n">
-        <v>1.153</v>
+        <v>2.948</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Uber</t>
+          <t>Shopee</t>
         </is>
       </c>
       <c r="M68" t="n">
-        <v>2.698</v>
+        <v>14.57</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>iFood Delivery de Comida</t>
+          <t>MercadoLibre</t>
         </is>
       </c>
       <c r="M69" t="n">
-        <v>2.157</v>
+        <v>5.876</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>99Taxis</t>
+          <t>SHEIN</t>
         </is>
       </c>
       <c r="M70" t="n">
-        <v>1.919</v>
+        <v>2.96</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>inDrive</t>
+          <t>AliExpress</t>
         </is>
       </c>
       <c r="M71" t="n">
-        <v>0.398</v>
+        <v>1.362</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Airbnb</t>
+          <t>Temu</t>
         </is>
       </c>
       <c r="M72" t="n">
-        <v>0.358</v>
+        <v>1.153</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
+          <t>Uber</t>
+        </is>
+      </c>
+      <c r="N74" t="n">
+        <v>2.698</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>iFood Delivery de Comida</t>
+        </is>
+      </c>
+      <c r="N75" t="n">
+        <v>2.157</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>99Taxis</t>
+        </is>
+      </c>
+      <c r="N76" t="n">
+        <v>1.919</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>inDrive</t>
+        </is>
+      </c>
+      <c r="N77" t="n">
+        <v>0.398</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Airbnb</t>
+        </is>
+      </c>
+      <c r="N78" t="n">
+        <v>0.358</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>ChatGPT</t>
+        </is>
+      </c>
+      <c r="O80" t="n">
+        <v>8.843999999999999</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Poly.AI - Create AI Chat Bot</t>
+        </is>
+      </c>
+      <c r="O81" t="n">
+        <v>8.096</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Emochi: Unlimited Chat with AI</t>
+        </is>
+      </c>
+      <c r="O82" t="n">
+        <v>4.556</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Character AI</t>
+        </is>
+      </c>
+      <c r="O83" t="n">
+        <v>3.288</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="O84" t="n">
+        <v>0.749</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
           <t>其他</t>
         </is>
       </c>
-      <c r="B74" t="n">
-        <v>18.22</v>
-      </c>
-      <c r="E74" t="n">
-        <v>3.73</v>
-      </c>
-      <c r="G74" t="n">
+      <c r="B86" t="n">
+        <v>17.584</v>
+      </c>
+      <c r="E86" t="n">
+        <v>2.316</v>
+      </c>
+      <c r="F86" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H86" t="n">
         <v>0.24</v>
       </c>
-      <c r="H74" t="n">
-        <v>2.824</v>
-      </c>
-      <c r="I74" t="n">
+      <c r="I86" t="n">
+        <v>2.789</v>
+      </c>
+      <c r="J86" t="n">
         <v>4.03</v>
       </c>
-      <c r="J74" t="n">
-        <v>4.683</v>
-      </c>
-      <c r="K74" t="n">
+      <c r="K86" t="n">
+        <v>4.639</v>
+      </c>
+      <c r="L86" t="n">
         <v>60.895</v>
       </c>
-      <c r="L74" t="n">
+      <c r="M86" t="n">
         <v>4.249</v>
       </c>
-      <c r="M74" t="n">
+      <c r="N86" t="n">
         <v>0.272</v>
+      </c>
+      <c r="O86" t="n">
+        <v>2.086</v>
       </c>
     </row>
   </sheetData>
@@ -1176,7 +1300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B54"/>
+  <dimension ref="A1:B49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1218,510 +1342,460 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ChatGPT</t>
+          <t>POCO Launcher 2.0 - Customize,</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8.843999999999999</v>
+        <v>6.581</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Poly.AI - Create AI Chat Bot</t>
+          <t>Google Maps</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8.096</v>
+        <v>5.412</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>POCO Launcher 2.0 - Customize,</t>
+          <t>Phone by Google</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6.581</v>
+        <v>5.011</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>Uber Driver</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5.412</v>
+        <v>3.547</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Phone by Google</t>
+          <t>Nubank</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5.011</v>
+        <v>3.401</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Emochi: Unlimited Chat with AI</t>
+          <t>OiTube</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4.556</v>
+        <v>3.071</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Uber Driver</t>
+          <t>YouTube Kids</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3.547</v>
+        <v>3.025</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Nubank</t>
+          <t>99 POP</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3.401</v>
+        <v>2.907</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Character AI</t>
+          <t>Duolingo: Learn Languages</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3.288</v>
+        <v>2.667</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>OiTube</t>
+          <t>Tomato - A&amp;M</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3.071</v>
+        <v>2.468</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>YouTube Kids</t>
+          <t>Itaú</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3.025</v>
+        <v>2.278</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>99 POP</t>
+          <t>ibisPaint</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2.907</v>
+        <v>2.183</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Duolingo: Learn Languages</t>
+          <t>Google Drive</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2.667</v>
+        <v>1.994</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Tomato - A&amp;M</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2.468</v>
+        <v>1.898</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Itaú</t>
+          <t>Samsung Clock</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2.278</v>
+        <v>1.752</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ibisPaint</t>
+          <t>Banco do Brasil</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2.183</v>
+        <v>1.457</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Google Drive</t>
+          <t>CAIXA</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1.994</v>
+        <v>1.457</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>Calculator by Google</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1.898</v>
+        <v>1.442</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Samsung Clock</t>
+          <t>Microsoft Teams</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1.752</v>
+        <v>1.374</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Banco do Brasil</t>
+          <t>Mercado Pago</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1.457</v>
+        <v>1.338</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAIXA</t>
+          <t>SnapTube</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1.457</v>
+        <v>1.241</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Calculator by Google</t>
+          <t>Crunchyroll</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1.442</v>
+        <v>1.198</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Microsoft Teams</t>
+          <t>Files Go by Google</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1.374</v>
+        <v>1.166</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>Bradesco</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1.338</v>
+        <v>1.103</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SnapTube</t>
+          <t>Santander Brasil</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1.241</v>
+        <v>1.059</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Crunchyroll</t>
+          <t>GreenTuber block ads on videos</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1.198</v>
+        <v>1.053</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Files Go by Google</t>
+          <t>Banco Inter</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1.166</v>
+        <v>1.013</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Bradesco</t>
+          <t>PicPay</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1.103</v>
+        <v>1.003</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Santander Brasil</t>
+          <t>Google Play services</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1.059</v>
+        <v>0.975</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GreenTuber block ads on videos</t>
+          <t>Canva</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1.053</v>
+        <v>0.914</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Banco Inter</t>
+          <t>Microsoft Outlook</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1.013</v>
+        <v>0.885</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>PicPay</t>
+          <t>Nova Launcher</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1.003</v>
+        <v>0.872</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Google Play services</t>
+          <t>FordBrowser</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.975</v>
+        <v>0.732</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Canva</t>
+          <t>Adobe Reader</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.914</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Microsoft Outlook</t>
+          <t>Samsung Calculator</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.885</v>
+        <v>0.653</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Nova Launcher</t>
+          <t>ZOOM Cloud Meetings</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.872</v>
+        <v>0.621</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>DeepSeek</t>
+          <t>Google Go</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.749</v>
+        <v>0.615</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>FordBrowser</t>
+          <t>Samsung Notes</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.732</v>
+        <v>0.609</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Adobe Reader</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.71</v>
+        <v>0.601</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Samsung Calculator</t>
+          <t>File Manager by  Flashlight Clock</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.653</v>
+        <v>0.587</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ZOOM Cloud Meetings</t>
+          <t>Google Docs</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.621</v>
+        <v>0.584</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Google Go</t>
+          <t>iCSee</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.615</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Samsung Notes</t>
+          <t>CineVS Oficial Filmes e Séries</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.609</v>
+        <v>0.5669999999999999</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>AnmBR</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.601</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>File Manager by  Flashlight Clock</t>
+          <t>Zapéx</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.587</v>
+        <v>0.547</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Google Docs</t>
+          <t>Glance</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0.584</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>iCSee</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>0.58</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>CineVS Oficial Filmes e Séries</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>0.5669999999999999</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>AnmBR</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Zapéx</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
-        <v>0.547</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Glance</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
         <v>0.522</v>
       </c>
     </row>

</xml_diff>